<commit_message>
update User Sign In,forgotpassword,endpoinds.properties and Testdata sheet
</commit_message>
<xml_diff>
--- a/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
+++ b/src/test/resources/Team01_RestAssured_Rebels_TestDataSheet.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Batch" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Program" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="User" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="ForgotPassword" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Batch" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Program" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="User" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="82">
   <si>
     <t xml:space="preserve">ScenarioName</t>
   </si>
@@ -43,6 +44,11 @@
     <t xml:space="preserve">Valid credential</t>
   </si>
   <si>
+    <t xml:space="preserve">{
+"userLoginEmailId":"VALID_EMAIL", "password":"VALID_PASS"
+}</t>
+  </si>
+  <si>
     <t xml:space="preserve">Invalid method</t>
   </si>
   <si>
@@ -59,8 +65,8 @@
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":"",
-"password":"adm123"
+"userLoginEmailId":"", 
+"password":"VALID_PASS"
 }</t>
   </si>
   <si>
@@ -68,8 +74,8 @@
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":"@#$",
-"password":"x"
+"userLoginEmailId":"@#$VALID_EMAIL", 
+"password":"VALID_PASS"
 }</t>
   </si>
   <si>
@@ -77,18 +83,15 @@
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":"test @gmail.com",
-"password":"12345"
-}
-</t>
+"userLoginEmailId":" VALID_EMAIL", "password":"VALID_PASS"}</t>
   </si>
   <si>
     <t xml:space="preserve">Null in email field</t>
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":null,
-"password":"aqwerp123"
+"userLoginEmailId":null, 
+"password":"VALID_PASS"
 }</t>
   </si>
   <si>
@@ -96,8 +99,7 @@
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":"pasha.12@gmail.com",
-"password":"adm123"
+"userLoginEmailId":"pasha.12@gmail.com", "password":"VALID_PASS"
 }</t>
   </si>
   <si>
@@ -105,7 +107,7 @@
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":"Team01@gmail.com",
+"userLoginEmailId":"VALID_EMAIL", 
 "password":" "
 }</t>
   </si>
@@ -114,8 +116,7 @@
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":"Team01@gmail.com",
-"password":"Abc@1234$"
+"userLoginEmailId":"VALID_EMAIL", "password":"#@VALID_PASS"
 }</t>
   </si>
   <si>
@@ -123,8 +124,8 @@
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":"Team01@gmail.com",
-"password":"adm 123"
+"userLoginEmailId":"VALID_EMAIL",
+ "password":"VALID_PASS  "
 }</t>
   </si>
   <si>
@@ -132,7 +133,7 @@
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":"Team01@gmail.com",
+"userLoginEmailId":"VALID_EMAIL", 
 "password":null
 }</t>
   </si>
@@ -141,12 +142,54 @@
   </si>
   <si>
     <t xml:space="preserve">{
-"userLoginEmailId":"inactive@gmail.com",
-"password":"inactive123"
+"userLoginEmailId":"inactive@gmail.com", "password":"inactive123"
 }</t>
   </si>
   <si>
     <t xml:space="preserve">Without request body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+"userLoginEmailId":"VALID_EMAIL"
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">But Given gherkin has 200 status code. 
+201 status API sends email for reset password 
+Request</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+"userLoginEmailId":"VALID_EMAIL"}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+"userLoginEmailId":""
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+"userLoginEmailId":"Ev@@gmail.com"
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Null email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+{"userLoginEmailId":null}
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+"userLoginEmailId":"admin.12@gmail.com"
+}</t>
   </si>
   <si>
     <t xml:space="preserve">CreateBatch_Valid_batchName</t>
@@ -403,7 +446,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,6 +477,19 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -456,14 +512,13 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -530,7 +585,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -542,24 +597,44 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -570,7 +645,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -578,31 +653,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -807,7 +862,7 @@
   <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="44.46"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.12"/>
@@ -833,11 +888,13 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="51.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="n">
         <v>200</v>
@@ -848,7 +905,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -861,7 +918,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -874,7 +931,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="2"/>
@@ -887,7 +944,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -900,10 +957,10 @@
     </row>
     <row r="7" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="3" t="s">
         <v>11</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="n">
@@ -913,12 +970,12 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="42.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="4" t="s">
         <v>13</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>14</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="n">
@@ -928,12 +985,12 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="33.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="3" t="s">
         <v>15</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="n">
@@ -944,11 +1001,11 @@
       <c r="G9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="3" t="s">
+      <c r="A10" s="8" t="s">
         <v>17</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2" t="n">
@@ -959,11 +1016,11 @@
       <c r="G10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>19</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>20</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="n">
@@ -974,11 +1031,11 @@
       <c r="G11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>21</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="n">
@@ -990,10 +1047,10 @@
     </row>
     <row r="13" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="9" t="s">
         <v>23</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>24</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="n">
@@ -1005,10 +1062,10 @@
     </row>
     <row r="14" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="3" t="s">
         <v>25</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2" t="n">
@@ -1020,10 +1077,10 @@
     </row>
     <row r="15" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="9" t="s">
         <v>27</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>28</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2" t="n">
@@ -1035,10 +1092,10 @@
     </row>
     <row r="16" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="9" t="s">
         <v>29</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>30</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2" t="n">
@@ -1050,7 +1107,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1153,7 +1210,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
-      <c r="B28" s="3"/>
+      <c r="B28" s="9"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1171,7 +1228,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
-      <c r="B30" s="3"/>
+      <c r="B30" s="9"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1199,7 +1256,7 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="10"/>
+      <c r="C33" s="12"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
@@ -9945,14 +10002,6 @@
       <c r="G1004" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B11" r:id="rId1" display="pasha.12@gmail.com"/>
-    <hyperlink ref="B12" r:id="rId2" display="Team01@gmail.com"/>
-    <hyperlink ref="B13" r:id="rId3" display="Team01@gmail.com"/>
-    <hyperlink ref="B14" r:id="rId4" display="Team01@gmail.com"/>
-    <hyperlink ref="B15" r:id="rId5" display="Team01@gmail.com"/>
-    <hyperlink ref="B16" r:id="rId6" display="inactive@gmail.com"/>
-  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -9968,161 +10017,128 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="11" width="36.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="33.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="11" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="11" width="19.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="11" width="14.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="33.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="35.35"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="11" t="s">
+      <c r="C1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="D1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-    </row>
-    <row r="2" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="13" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="33.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="B2" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="11" t="n">
+      <c r="C2" s="0" t="n">
         <v>201</v>
       </c>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-    </row>
-    <row r="3" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="E2" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="13" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="21.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="0" t="n">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="32.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="16" t="n">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
+      <c r="C5" s="0" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="33.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="C6" s="0" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="32.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="16" t="n">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="83.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
+      <c r="B7" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="C7" s="0" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="32.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="16" t="n">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
+      <c r="B8" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="C8" s="0" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="33.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="16" t="n">
+      <c r="C9" s="0" t="n">
         <v>400</v>
       </c>
-      <c r="E6" s="17" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="21" t="n">
-        <v>401</v>
-      </c>
-      <c r="E7" s="0"/>
-    </row>
-    <row r="8" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="21" t="n">
-        <v>400</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>46</v>
-      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B9" r:id="rId1" display="admin.12@gmail.com"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -10132,121 +10148,152 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="11" width="12.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="27.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="16" width="36.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="16" width="33.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="16" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="16" width="19.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="16" width="14.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+    </row>
+    <row r="2" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="16" t="n">
+        <v>201</v>
+      </c>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+    </row>
+    <row r="3" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="21" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="12"/>
-      <c r="S1" s="12"/>
-      <c r="T1" s="12"/>
-      <c r="U1" s="12"/>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="12"/>
-      <c r="Z1" s="12"/>
-    </row>
-    <row r="2" customFormat="false" ht="142.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
+      <c r="B4" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="C4" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="83.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="B5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="C5" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="12" t="n">
-        <v>201</v>
-      </c>
-      <c r="F2" s="12" t="s">
+      <c r="B6" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
-      <c r="V2" s="12"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="12"/>
-      <c r="Z2" s="12"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
-      <c r="V3" s="12"/>
-      <c r="W3" s="12"/>
-      <c r="X3" s="12"/>
-      <c r="Y3" s="12"/>
-      <c r="Z3" s="12"/>
+      <c r="C6" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="73.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>57</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -10260,6 +10307,138 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:Z3"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="16" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="16" width="12.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="16" width="27.03"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
+      <c r="T1" s="17"/>
+      <c r="U1" s="17"/>
+      <c r="V1" s="17"/>
+      <c r="W1" s="17"/>
+      <c r="X1" s="17"/>
+      <c r="Y1" s="17"/>
+      <c r="Z1" s="17"/>
+    </row>
+    <row r="2" customFormat="false" ht="142.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="E2" s="17" t="n">
+        <v>201</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="17"/>
+      <c r="V2" s="17"/>
+      <c r="W2" s="17"/>
+      <c r="X2" s="17"/>
+      <c r="Y2" s="17"/>
+      <c r="Z2" s="17"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="17"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="17"/>
+      <c r="O3" s="17"/>
+      <c r="P3" s="17"/>
+      <c r="Q3" s="17"/>
+      <c r="R3" s="17"/>
+      <c r="S3" s="17"/>
+      <c r="T3" s="17"/>
+      <c r="U3" s="17"/>
+      <c r="V3" s="17"/>
+      <c r="W3" s="17"/>
+      <c r="X3" s="17"/>
+      <c r="Y3" s="17"/>
+      <c r="Z3" s="17"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -10282,21 +10461,21 @@
         <v>1</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="261.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D2" s="22" t="n">
         <v>201</v>
@@ -10304,13 +10483,13 @@
     </row>
     <row r="3" customFormat="false" ht="272.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D3" s="23" t="n">
         <v>201</v>
@@ -10318,13 +10497,13 @@
     </row>
     <row r="4" customFormat="false" ht="261.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D4" s="23" t="n">
         <v>201</v>
@@ -10332,71 +10511,71 @@
     </row>
     <row r="5" customFormat="false" ht="207.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="D5" s="23" t="n">
         <v>201</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" s="7" t="n">
+      <c r="A6" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" s="7" t="n">
+      <c r="A7" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>404</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="7" t="n">
+      <c r="A8" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" s="4" t="n">
         <v>405</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" s="7" t="n">
+      <c r="A9" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" s="4" t="n">
         <v>401</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>